<commit_message>
fix: lieu de formation en CodeableConcept lié à JDV-J235-LieuFormation-EPARS (#315)
* fix: lieu de formation en CodeableConcept lié à JDV-J235-LieuFormation-EPARS

Remplace la Reference(Organization) de qualification[degree].issuer par
une sous-extension CodeableConcept dans AsEducationLevelExtension, pour
décrire le type de lieu ayant délivré le diplôme plutôt qu'une
organisation précise.

Fixes #314

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>

* docs: référence le numéro de PR #315 dans le changelog

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>

---------

Co-authored-by: Claude Sonnet 5 <noreply@anthropic.com> 0bb967da04b249fc4d8d630f4ec41eb04c8c9d8c
</commit_message>
<xml_diff>
--- a/main/ig/StructureDefinition-as-ext-education-level.xlsx
+++ b/main/ig/StructureDefinition-as-ext-education-level.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="721" uniqueCount="143">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="882" uniqueCount="151">
   <si>
     <t>Property</t>
   </si>
@@ -57,7 +57,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-06-30T07:59:11+00:00</t>
+    <t>2026-07-10T15:33:23+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -450,6 +450,30 @@
   </si>
   <si>
     <t>https://mos.esante.gouv.fr/NOS/JDV_J88-AnneeUniversitaire-RASS/FHIR/JDV-J88-AnneeUniversitaire-RASS|20251016120000</t>
+  </si>
+  <si>
+    <t>Extension.extension:trainingLocation</t>
+  </si>
+  <si>
+    <t>trainingLocation</t>
+  </si>
+  <si>
+    <t>[Donnée restreinte] : Type de lieu ayant délivré le diplôme (lieuFormation).</t>
+  </si>
+  <si>
+    <t>Extension.extension:trainingLocation.id</t>
+  </si>
+  <si>
+    <t>Extension.extension:trainingLocation.extension</t>
+  </si>
+  <si>
+    <t>Extension.extension:trainingLocation.url</t>
+  </si>
+  <si>
+    <t>Extension.extension:trainingLocation.value[x]</t>
+  </si>
+  <si>
+    <t>https://mos.esante.gouv.fr/NOS/JDV_J235-LieuFormation-EPARS/FHIR/JDV-J235-LieuFormation-EPARS|20240726120000</t>
   </si>
   <si>
     <t>base64Binary
@@ -763,7 +787,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:AK21"/>
+  <dimension ref="A1:AK26"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <cols>
     <col min="1" max="1" width="38.86328125" customWidth="true" bestFit="true"/>
@@ -2781,18 +2805,20 @@
     </row>
     <row r="20">
       <c r="A20" t="s" s="2">
-        <v>115</v>
+        <v>142</v>
       </c>
       <c r="B20" t="s" s="2">
-        <v>115</v>
-      </c>
-      <c r="C20" s="2"/>
+        <v>91</v>
+      </c>
+      <c r="C20" t="s" s="2">
+        <v>143</v>
+      </c>
       <c r="D20" t="s" s="2">
         <v>76</v>
       </c>
       <c r="E20" s="2"/>
       <c r="F20" t="s" s="2">
-        <v>85</v>
+        <v>77</v>
       </c>
       <c r="G20" t="s" s="2">
         <v>85</v>
@@ -2807,24 +2833,22 @@
         <v>76</v>
       </c>
       <c r="K20" t="s" s="2">
-        <v>111</v>
+        <v>93</v>
       </c>
       <c r="L20" t="s" s="2">
-        <v>112</v>
+        <v>144</v>
       </c>
       <c r="M20" t="s" s="2">
-        <v>113</v>
-      </c>
-      <c r="N20" t="s" s="2">
-        <v>114</v>
-      </c>
+        <v>104</v>
+      </c>
+      <c r="N20" s="2"/>
       <c r="O20" s="2"/>
       <c r="P20" t="s" s="2">
         <v>76</v>
       </c>
       <c r="Q20" s="2"/>
       <c r="R20" t="s" s="2">
-        <v>3</v>
+        <v>76</v>
       </c>
       <c r="S20" t="s" s="2">
         <v>76</v>
@@ -2866,30 +2890,30 @@
         <v>76</v>
       </c>
       <c r="AF20" t="s" s="2">
-        <v>115</v>
+        <v>100</v>
       </c>
       <c r="AG20" t="s" s="2">
-        <v>85</v>
+        <v>77</v>
       </c>
       <c r="AH20" t="s" s="2">
-        <v>85</v>
+        <v>78</v>
       </c>
       <c r="AI20" t="s" s="2">
         <v>76</v>
       </c>
       <c r="AJ20" t="s" s="2">
-        <v>76</v>
+        <v>83</v>
       </c>
       <c r="AK20" t="s" s="2">
-        <v>116</v>
+        <v>76</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="s" s="2">
-        <v>124</v>
+        <v>145</v>
       </c>
       <c r="B21" t="s" s="2">
-        <v>124</v>
+        <v>106</v>
       </c>
       <c r="C21" s="2"/>
       <c r="D21" t="s" s="2">
@@ -2900,7 +2924,7 @@
         <v>77</v>
       </c>
       <c r="G21" t="s" s="2">
-        <v>77</v>
+        <v>85</v>
       </c>
       <c r="H21" t="s" s="2">
         <v>76</v>
@@ -2912,13 +2936,13 @@
         <v>76</v>
       </c>
       <c r="K21" t="s" s="2">
-        <v>142</v>
+        <v>86</v>
       </c>
       <c r="L21" t="s" s="2">
-        <v>120</v>
+        <v>87</v>
       </c>
       <c r="M21" t="s" s="2">
-        <v>121</v>
+        <v>88</v>
       </c>
       <c r="N21" s="2"/>
       <c r="O21" s="2"/>
@@ -2969,21 +2993,538 @@
         <v>76</v>
       </c>
       <c r="AF21" t="s" s="2">
+        <v>89</v>
+      </c>
+      <c r="AG21" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AH21" t="s" s="2">
+        <v>85</v>
+      </c>
+      <c r="AI21" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AJ21" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AK21" t="s" s="2">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="s" s="2">
+        <v>146</v>
+      </c>
+      <c r="B22" t="s" s="2">
+        <v>108</v>
+      </c>
+      <c r="C22" s="2"/>
+      <c r="D22" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="E22" s="2"/>
+      <c r="F22" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="G22" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="H22" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="I22" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="J22" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="K22" t="s" s="2">
+        <v>93</v>
+      </c>
+      <c r="L22" t="s" s="2">
+        <v>30</v>
+      </c>
+      <c r="M22" t="s" s="2">
+        <v>104</v>
+      </c>
+      <c r="N22" s="2"/>
+      <c r="O22" s="2"/>
+      <c r="P22" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="Q22" s="2"/>
+      <c r="R22" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="S22" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="T22" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="U22" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="V22" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="W22" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="X22" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="Y22" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="Z22" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AA22" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AB22" t="s" s="2">
+        <v>97</v>
+      </c>
+      <c r="AC22" t="s" s="2">
+        <v>98</v>
+      </c>
+      <c r="AD22" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AE22" t="s" s="2">
+        <v>99</v>
+      </c>
+      <c r="AF22" t="s" s="2">
+        <v>100</v>
+      </c>
+      <c r="AG22" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AH22" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="AI22" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AJ22" t="s" s="2">
+        <v>83</v>
+      </c>
+      <c r="AK22" t="s" s="2">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="s" s="2">
+        <v>147</v>
+      </c>
+      <c r="B23" t="s" s="2">
+        <v>110</v>
+      </c>
+      <c r="C23" s="2"/>
+      <c r="D23" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="E23" s="2"/>
+      <c r="F23" t="s" s="2">
+        <v>85</v>
+      </c>
+      <c r="G23" t="s" s="2">
+        <v>85</v>
+      </c>
+      <c r="H23" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="I23" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="J23" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="K23" t="s" s="2">
+        <v>111</v>
+      </c>
+      <c r="L23" t="s" s="2">
+        <v>112</v>
+      </c>
+      <c r="M23" t="s" s="2">
+        <v>113</v>
+      </c>
+      <c r="N23" t="s" s="2">
+        <v>114</v>
+      </c>
+      <c r="O23" s="2"/>
+      <c r="P23" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="Q23" s="2"/>
+      <c r="R23" t="s" s="2">
+        <v>143</v>
+      </c>
+      <c r="S23" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="T23" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="U23" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="V23" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="W23" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="X23" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="Y23" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="Z23" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AA23" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AB23" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AC23" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AD23" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AE23" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AF23" t="s" s="2">
+        <v>115</v>
+      </c>
+      <c r="AG23" t="s" s="2">
+        <v>85</v>
+      </c>
+      <c r="AH23" t="s" s="2">
+        <v>85</v>
+      </c>
+      <c r="AI23" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AJ23" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AK23" t="s" s="2">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="s" s="2">
+        <v>148</v>
+      </c>
+      <c r="B24" t="s" s="2">
+        <v>118</v>
+      </c>
+      <c r="C24" s="2"/>
+      <c r="D24" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="E24" s="2"/>
+      <c r="F24" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="G24" t="s" s="2">
+        <v>85</v>
+      </c>
+      <c r="H24" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="I24" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="J24" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="K24" t="s" s="2">
+        <v>119</v>
+      </c>
+      <c r="L24" t="s" s="2">
+        <v>120</v>
+      </c>
+      <c r="M24" t="s" s="2">
+        <v>121</v>
+      </c>
+      <c r="N24" s="2"/>
+      <c r="O24" s="2"/>
+      <c r="P24" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="Q24" s="2"/>
+      <c r="R24" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="S24" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="T24" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="U24" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="V24" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="W24" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="X24" t="s" s="2">
+        <v>122</v>
+      </c>
+      <c r="Y24" s="2"/>
+      <c r="Z24" t="s" s="2">
+        <v>149</v>
+      </c>
+      <c r="AA24" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AB24" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AC24" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AD24" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AE24" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AF24" t="s" s="2">
         <v>124</v>
       </c>
-      <c r="AG21" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="AH21" t="s" s="2">
-        <v>85</v>
-      </c>
-      <c r="AI21" t="s" s="2">
-        <v>76</v>
-      </c>
-      <c r="AJ21" t="s" s="2">
+      <c r="AG24" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AH24" t="s" s="2">
+        <v>85</v>
+      </c>
+      <c r="AI24" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AJ24" t="s" s="2">
         <v>125</v>
       </c>
-      <c r="AK21" t="s" s="2">
+      <c r="AK24" t="s" s="2">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="s" s="2">
+        <v>115</v>
+      </c>
+      <c r="B25" t="s" s="2">
+        <v>115</v>
+      </c>
+      <c r="C25" s="2"/>
+      <c r="D25" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="E25" s="2"/>
+      <c r="F25" t="s" s="2">
+        <v>85</v>
+      </c>
+      <c r="G25" t="s" s="2">
+        <v>85</v>
+      </c>
+      <c r="H25" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="I25" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="J25" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="K25" t="s" s="2">
+        <v>111</v>
+      </c>
+      <c r="L25" t="s" s="2">
+        <v>112</v>
+      </c>
+      <c r="M25" t="s" s="2">
+        <v>113</v>
+      </c>
+      <c r="N25" t="s" s="2">
+        <v>114</v>
+      </c>
+      <c r="O25" s="2"/>
+      <c r="P25" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="Q25" s="2"/>
+      <c r="R25" t="s" s="2">
+        <v>3</v>
+      </c>
+      <c r="S25" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="T25" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="U25" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="V25" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="W25" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="X25" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="Y25" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="Z25" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AA25" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AB25" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AC25" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AD25" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AE25" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AF25" t="s" s="2">
+        <v>115</v>
+      </c>
+      <c r="AG25" t="s" s="2">
+        <v>85</v>
+      </c>
+      <c r="AH25" t="s" s="2">
+        <v>85</v>
+      </c>
+      <c r="AI25" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AJ25" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AK25" t="s" s="2">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="s" s="2">
+        <v>124</v>
+      </c>
+      <c r="B26" t="s" s="2">
+        <v>124</v>
+      </c>
+      <c r="C26" s="2"/>
+      <c r="D26" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="E26" s="2"/>
+      <c r="F26" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="G26" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="H26" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="I26" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="J26" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="K26" t="s" s="2">
+        <v>150</v>
+      </c>
+      <c r="L26" t="s" s="2">
+        <v>120</v>
+      </c>
+      <c r="M26" t="s" s="2">
+        <v>121</v>
+      </c>
+      <c r="N26" s="2"/>
+      <c r="O26" s="2"/>
+      <c r="P26" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="Q26" s="2"/>
+      <c r="R26" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="S26" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="T26" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="U26" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="V26" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="W26" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="X26" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="Y26" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="Z26" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AA26" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AB26" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AC26" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AD26" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AE26" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AF26" t="s" s="2">
+        <v>124</v>
+      </c>
+      <c r="AG26" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AH26" t="s" s="2">
+        <v>85</v>
+      </c>
+      <c r="AI26" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AJ26" t="s" s="2">
+        <v>125</v>
+      </c>
+      <c r="AK26" t="s" s="2">
         <v>116</v>
       </c>
     </row>

</xml_diff>